<commit_message>
ref: change other files
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Новая папка\Uni 2 course  1 semestr\КГВ\STEM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B91E0567-4D86-44CA-B211-0F3360FAC228}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D3F0256-F532-4F1B-A05E-31399A903FAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3604,6 +3604,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AA842"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A1" t="s">

</xml_diff>